<commit_message>
da do dung du lieu vao tung cot
</commit_message>
<xml_diff>
--- a/app-templates/users (21).xlsx
+++ b/app-templates/users (21).xlsx
@@ -11,10 +11,11 @@
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="NgayLabel">Export!$C$4</definedName>
+    <definedName name="NgayLabel">Export!$F$4</definedName>
     <definedName name="ngayValue">Export!$F$4</definedName>
-    <definedName name="header">Export!$C$8:$AI$8</definedName>
-    <definedName name="value">Export!$C$9:$AI$9</definedName>
+    <definedName name="han">Export!$C$9</definedName>
+    <definedName name="ten">Export!$K$9</definedName>
+    <definedName name="so">Export!$P$9</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>